<commit_message>
updated readme and update tracker
</commit_message>
<xml_diff>
--- a/Enterprise_Project_Planner_v4.xlsx
+++ b/Enterprise_Project_Planner_v4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\Desktop\Workspace\ai-auto-healing-platform\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\Desktop\Workspace\Multi-Cloud-Kubernetes-Auto-Healing-Auto-Scaling-Platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54BF19BE-52F5-4D1D-A0FC-596DE16C6754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF28171-F59F-4D99-86E2-BDB4F0BEC26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Dashboard" sheetId="1" r:id="rId1"/>
@@ -21,14 +21,13 @@
     <sheet name="RAID Log" sheetId="6" r:id="rId6"/>
     <sheet name="Milestone Tracker" sheetId="7" r:id="rId7"/>
     <sheet name="Weekly Status Report" sheetId="8" r:id="rId8"/>
-    <sheet name="Resume Tracker" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="111">
   <si>
     <t>Metric</t>
   </si>
@@ -90,9 +89,6 @@
     <t>Infrastructure</t>
   </si>
   <si>
-    <t>Terraform, AWS EKS, Azure AKS, IAM, Networking</t>
-  </si>
-  <si>
     <t>Not Started</t>
   </si>
   <si>
@@ -360,20 +356,17 @@
     <t>Next Week Plan</t>
   </si>
   <si>
-    <t>Area</t>
-  </si>
-  <si>
-    <t>Achievement</t>
-  </si>
-  <si>
-    <t>Resume Bullet</t>
+    <t>https://github.com/vkharishb/Multi-Cloud-Kubernetes-Auto-Healing-Auto-Scaling-Platform.git</t>
+  </si>
+  <si>
+    <t>Terraform, AWS EKS, Azure AKS, IAM, Networking, Git</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -385,6 +378,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -404,10 +405,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -416,11 +418,49 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -829,55 +869,60 @@
         <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{F96AF115-EBE9-4D30-9D0B-922FF8F5B5EE}">
+      <formula1>"Not Started,In Progress,Blocked,Completed,Deferred"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -890,30 +935,31 @@
     <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
+    <col min="7" max="7" width="79.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -924,16 +970,19 @@
         <v>18</v>
       </c>
       <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
         <v>36</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
       </c>
       <c r="E2">
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>106</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -944,16 +993,16 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
         <v>38</v>
-      </c>
-      <c r="D3" t="s">
-        <v>39</v>
       </c>
       <c r="E3">
         <v>6</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -964,16 +1013,16 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
         <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
       </c>
       <c r="E4">
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -984,16 +1033,16 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
         <v>42</v>
-      </c>
-      <c r="D5" t="s">
-        <v>43</v>
       </c>
       <c r="E5">
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1004,16 +1053,16 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
         <v>44</v>
-      </c>
-      <c r="D6" t="s">
-        <v>45</v>
       </c>
       <c r="E6">
         <v>6</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -1024,16 +1073,16 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E7">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -1044,16 +1093,16 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
         <v>47</v>
-      </c>
-      <c r="D8" t="s">
-        <v>48</v>
       </c>
       <c r="E8">
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -1061,19 +1110,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
         <v>49</v>
-      </c>
-      <c r="D9" t="s">
-        <v>50</v>
       </c>
       <c r="E9">
         <v>6</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1081,19 +1130,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -1101,19 +1150,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
         <v>52</v>
-      </c>
-      <c r="D11" t="s">
-        <v>53</v>
       </c>
       <c r="E11">
         <v>6</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -1121,19 +1170,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
         <v>54</v>
-      </c>
-      <c r="D12" t="s">
-        <v>55</v>
       </c>
       <c r="E12">
         <v>6</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1141,19 +1190,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
         <v>56</v>
-      </c>
-      <c r="D13" t="s">
-        <v>57</v>
       </c>
       <c r="E13">
         <v>6</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1161,19 +1210,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
         <v>58</v>
-      </c>
-      <c r="D14" t="s">
-        <v>59</v>
       </c>
       <c r="E14">
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -1181,19 +1230,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" t="s">
         <v>60</v>
-      </c>
-      <c r="D15" t="s">
-        <v>61</v>
       </c>
       <c r="E15">
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1201,19 +1250,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" t="s">
         <v>62</v>
-      </c>
-      <c r="D16" t="s">
-        <v>63</v>
       </c>
       <c r="E16">
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1221,19 +1270,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" t="s">
         <v>64</v>
-      </c>
-      <c r="D17" t="s">
-        <v>65</v>
       </c>
       <c r="E17">
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1241,19 +1290,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" t="s">
         <v>66</v>
-      </c>
-      <c r="D18" t="s">
-        <v>67</v>
       </c>
       <c r="E18">
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1261,19 +1310,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" t="s">
         <v>68</v>
-      </c>
-      <c r="D19" t="s">
-        <v>69</v>
       </c>
       <c r="E19">
         <v>6</v>
       </c>
       <c r="F19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1281,19 +1330,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" t="s">
         <v>70</v>
-      </c>
-      <c r="D20" t="s">
-        <v>71</v>
       </c>
       <c r="E20">
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1301,19 +1350,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" t="s">
         <v>72</v>
-      </c>
-      <c r="D21" t="s">
-        <v>73</v>
       </c>
       <c r="E21">
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1321,19 +1370,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" t="s">
         <v>74</v>
-      </c>
-      <c r="D22" t="s">
-        <v>75</v>
       </c>
       <c r="E22">
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1341,19 +1390,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" t="s">
         <v>76</v>
-      </c>
-      <c r="D23" t="s">
-        <v>77</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1361,19 +1410,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" t="s">
         <v>78</v>
-      </c>
-      <c r="D24" t="s">
-        <v>79</v>
       </c>
       <c r="E24">
         <v>3</v>
       </c>
       <c r="F24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1381,19 +1430,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" t="s">
         <v>80</v>
-      </c>
-      <c r="D25" t="s">
-        <v>81</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1401,19 +1450,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" t="s">
         <v>82</v>
-      </c>
-      <c r="D26" t="s">
-        <v>83</v>
       </c>
       <c r="E26">
         <v>6</v>
       </c>
       <c r="F26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1421,19 +1470,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" t="s">
         <v>84</v>
-      </c>
-      <c r="D27" t="s">
-        <v>85</v>
       </c>
       <c r="E27">
         <v>6</v>
       </c>
       <c r="F27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1441,19 +1490,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" t="s">
         <v>86</v>
-      </c>
-      <c r="D28" t="s">
-        <v>87</v>
       </c>
       <c r="E28">
         <v>2</v>
       </c>
       <c r="F28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1461,22 +1510,49 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C29" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" t="s">
         <v>88</v>
-      </c>
-      <c r="D29" t="s">
-        <v>89</v>
       </c>
       <c r="E29">
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:G2">
+    <cfRule type="cellIs" dxfId="4" priority="5" stopIfTrue="1" operator="equal">
+      <formula>"Deferred"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F1:F1048576 G2">
+    <cfRule type="cellIs" dxfId="3" priority="4" stopIfTrue="1" operator="equal">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="equal">
+      <formula>"Blocked "</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">
+      <formula>"Completed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F28" xr:uid="{88B4A230-DCAB-4671-9F6F-5A60A415E615}">
+      <formula1>"Not Started,In Progress,Blocked,Completed,Deferred"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{5F8FFB7B-27E4-4774-B0E8-E6D38E1B73D6}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1488,10 +1564,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>17</v>
@@ -1509,13 +1585,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
@@ -1533,13 +1609,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
@@ -1554,10 +1630,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1568,68 +1648,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
         <v>98</v>
       </c>
-      <c r="B2" t="s">
-        <v>99</v>
-      </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" t="s">
-        <v>102</v>
-      </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" t="s">
         <v>103</v>
       </c>
-      <c r="B5" t="s">
-        <v>104</v>
-      </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1641,43 +1721,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>